<commit_message>
feat: adicionando novas perguntas, controle automatico do csv, e pop-up sobre csv
</commit_message>
<xml_diff>
--- a/modelo-perguntas.xlsx
+++ b/modelo-perguntas.xlsx
@@ -2,41 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\Projetos Facul\Projeto TecnoMack\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projetos Facul\Projeto TecnoMack\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{22D8D3F4-B31F-4DDA-8D8A-14B2C2A9D709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FF78DAA-2982-4715-A1D7-4B82BCA817DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="15375" windowHeight="8325" xr2:uid="{6A1B4E4E-8A7E-47A2-AF57-CD48790BD675}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Perguntas" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="194">
   <si>
     <t>level</t>
   </si>
@@ -348,6 +332,276 @@
   </si>
   <si>
     <t>Não! Embora atualizações possam consumir recursos, a proteção vale a pena.</t>
+  </si>
+  <si>
+    <t>Qual é a principal função de um antivírus?</t>
+  </si>
+  <si>
+    <t>Deixar o computador mais rápido</t>
+  </si>
+  <si>
+    <t>Proteger o computador contra vírus e golpes pela internet</t>
+  </si>
+  <si>
+    <t>Guardar fotos e documentos</t>
+  </si>
+  <si>
+    <t>Aumentar o volume do som</t>
+  </si>
+  <si>
+    <t>Não, ele não serve para melhorar a velocidade.</t>
+  </si>
+  <si>
+    <t>Correto! O antivírus ajuda a proteger o computador contra vírus e ameaças.</t>
+  </si>
+  <si>
+    <t>Não, guardar arquivos é função de outros programas.</t>
+  </si>
+  <si>
+    <t>Não, isso não tem relação com segurança.</t>
+  </si>
+  <si>
+    <t>O que é a verificação em duas etapas (2FA)?</t>
+  </si>
+  <si>
+    <t>Receber um código no celular para confirmar o acesso</t>
+  </si>
+  <si>
+    <t>Usar a mesma senha duas vezes</t>
+  </si>
+  <si>
+    <t>Pedir ajuda para outra pessoa entrar na conta</t>
+  </si>
+  <si>
+    <t>Não usar senha</t>
+  </si>
+  <si>
+    <t>Correto! Além da senha, você recebe um código no celular para confirmar que é você.</t>
+  </si>
+  <si>
+    <t>Não, repetir a senha não aumenta a segurança.</t>
+  </si>
+  <si>
+    <t>Não, isso pode até ser perigoso.</t>
+  </si>
+  <si>
+    <t>Não, não usar senha deixa a conta vulnerável.</t>
+  </si>
+  <si>
+    <t>O que devo fazer ao receber um e-mail desconhecido pedindo para clicar em um link?</t>
+  </si>
+  <si>
+    <t>Clicar no link rapidamente para ver do que se trata</t>
+  </si>
+  <si>
+    <t>Ignorar completamente sem verificar nada</t>
+  </si>
+  <si>
+    <t>Copiar o link e verificar com cuidado antes de acessar</t>
+  </si>
+  <si>
+    <t>Encaminhar o e-mail para amigos</t>
+  </si>
+  <si>
+    <t>Não é seguro clicar em links desconhecidos, pois podem ser golpes para roubar seus dados.</t>
+  </si>
+  <si>
+    <t>Ignorar pode até evitar o risco, mas o ideal é saber identificar se é um golpe ou não.</t>
+  </si>
+  <si>
+    <t>Correto! Copiar e verificar o link com cuidado ajuda a evitar cair em golpes.</t>
+  </si>
+  <si>
+    <t>Encaminhar pode espalhar o golpe para outras pessoas. O melhor é não compartilhar.</t>
+  </si>
+  <si>
+    <t>Se você receber um e-mail dizendo ser de um órgão público cobrando uma pendência financeira e pedindo para clicar em um link para regularizar, o que você deve fazer?</t>
+  </si>
+  <si>
+    <t>Não clicar no link e buscar o site oficial do órgão para verificar a informação</t>
+  </si>
+  <si>
+    <t>Clicar no link rapidamente para evitar problemas no CPF</t>
+  </si>
+  <si>
+    <t>Responder o e-mail enviando seus dados pessoais</t>
+  </si>
+  <si>
+    <t>Ignorar o risco e confiar na mensagem recebida</t>
+  </si>
+  <si>
+    <t>Correto! Órgãos públicos não enviam cobranças com links por e-mail. O mais seguro é acessar o site oficial para verificar.</t>
+  </si>
+  <si>
+    <t>Clicar no link pode levar a páginas falsas criadas para roubar seus dados.</t>
+  </si>
+  <si>
+    <t>Enviar dados pessoais pode expor você a golpes e fraudes.</t>
+  </si>
+  <si>
+    <t>Ignorar o risco pode fazer você cair em um golpe. Sempre desconfie de mensagens desse tipo.</t>
+  </si>
+  <si>
+    <t>Você recebeu uma mensagem no WhatsApp de um número desconhecido dizendo que ganhou um prêmio e pedindo para clicar num link. O que você deve fazer?</t>
+  </si>
+  <si>
+    <t>Clicar no link para ver o prêmio</t>
+  </si>
+  <si>
+    <t>Encaminhar para os amigos verem também</t>
+  </si>
+  <si>
+    <t>Ignorar, apagar a mensagem e bloquear o número</t>
+  </si>
+  <si>
+    <t>Responder perguntando mais detalhes sobre o prêmio</t>
+  </si>
+  <si>
+    <t>Nunca clique em links de mensagens de desconhecidos! Esse é um golpe muito comum para roubar seus dados.</t>
+  </si>
+  <si>
+    <t>Ao encaminhar, você pode estar espalhando o golpe para seus amigos e familiares. Não compartilhe mensagens suspeitas.</t>
+  </si>
+  <si>
+    <t>Correto! Mensagens de prêmios de desconhecidos são quase sempre golpes. Apague e bloqueie o número.</t>
+  </si>
+  <si>
+    <t>Responder mostra que seu número está ativo, e você pode receber ainda mais mensagens de golpe.</t>
+  </si>
+  <si>
+    <t>Anota suas senhas num caderno virtual sem proteção</t>
+  </si>
+  <si>
+    <t>Guarda todas as suas senhas de forma segura e protegida</t>
+  </si>
+  <si>
+    <t>Compartilha suas senhas com outras pessoas</t>
+  </si>
+  <si>
+    <t>Deixa suas senhas visíveis para qualquer um no celular</t>
+  </si>
+  <si>
+    <t>Anotar senhas sem proteção é perigoso, pois qualquer pessoa com acesso ao seu dispositivo pode vê-las.</t>
+  </si>
+  <si>
+    <t>Correto! Aplicativos de guardar senhas (como o que vem no celular) protegem suas senhas com segurança e ajudam a criar senhas fortes.</t>
+  </si>
+  <si>
+    <t>Não, esses aplicativos não compartilham suas senhas. Só você tem acesso.</t>
+  </si>
+  <si>
+    <t>Não! Esses aplicativos protegem suas senhas com uma senha mestra ou pela digital do seu dedo.</t>
+  </si>
+  <si>
+    <t>Você percebeu que alguém entrou na sua conta de email sem sua permissão. O que você deve fazer primeiro?</t>
+  </si>
+  <si>
+    <t>Criar um novo email e esquecer o antigo</t>
+  </si>
+  <si>
+    <t>Trocar a senha do email o mais rápido possível</t>
+  </si>
+  <si>
+    <t>Esperar para ver se acontece algo de errado</t>
+  </si>
+  <si>
+    <t>Avisar seus amigos pelo mesmo email invadido</t>
+  </si>
+  <si>
+    <t>Criar um novo email pode ser necessário depois, mas primeiro tente recuperar o acesso trocando a senha rapidamente.</t>
+  </si>
+  <si>
+    <t>Correto! Troque a senha imediatamente. Depois, avise seus contatos para ignorarem mensagens estranhas que vieram do seu email.</t>
+  </si>
+  <si>
+    <t>Quanto mais tempo você espera, mais tempo a pessoa mal-intencionada tem para causar estragos.</t>
+  </si>
+  <si>
+    <t>Usar o email invadido para se comunicar é arriscado. A outra pessoa ainda pode estar vendo tudo. Troque a senha primeiro.</t>
+  </si>
+  <si>
+    <t>Qual a melhor forma de guardar cópias das suas fotos e documentos importantes?</t>
+  </si>
+  <si>
+    <t>Deixar tudo apenas no computador ou celular</t>
+  </si>
+  <si>
+    <t>Guardar somente num pen drive ou HD externo</t>
+  </si>
+  <si>
+    <t>Ter cópias em mais de um lugar: no aparelho, num pen drive e na nuvem</t>
+  </si>
+  <si>
+    <t>Fazer uma cópia por ano é suficiente</t>
+  </si>
+  <si>
+    <t>Se o computador ou celular estragar ou for roubado, você perde tudo. Sempre tenha cópias em outros lugares.</t>
+  </si>
+  <si>
+    <t>Melhor do que nada, mas pen drives e HDs também podem estragar ou se perder. Tenha mais de uma cópia.</t>
+  </si>
+  <si>
+    <t>Correto! O ideal é ter cópias em pelo menos dois ou três lugares diferentes. A nuvem (como Google Fotos ou iCloud) é ótima opção.</t>
+  </si>
+  <si>
+    <t>Fotos e documentos mudam o tempo todo. Faça cópias com frequência, especialmente de arquivos que você não quer perder nunca.</t>
+  </si>
+  <si>
+    <t>Quando você desbloqueia o celular com o seu rosto ou a impressão digital, o que está usando?</t>
+  </si>
+  <si>
+    <t>Uma senha muito complicada</t>
+  </si>
+  <si>
+    <t>Uma confirmação pelo celular de outra pessoa</t>
+  </si>
+  <si>
+    <t>Uma característica do seu próprio corpo como forma de identificação</t>
+  </si>
+  <si>
+    <t>Um método menos seguro do que uma senha simples</t>
+  </si>
+  <si>
+    <t>Não é uma senha. É o reconhecimento de uma parte do seu corpo, como o rosto ou a digital.</t>
+  </si>
+  <si>
+    <t>Não envolve outra pessoa. É você mesmo sendo reconhecido pelo aparelho.</t>
+  </si>
+  <si>
+    <t>Correto! Usar o rosto ou a digital é chamado de autenticação biométrica. É muito seguro porque é difícil de copiar.</t>
+  </si>
+  <si>
+    <t>Ao contrário! É mais seguro do que senhas simples, porque ninguém consegue copiar o seu rosto ou sua digital facilmente.</t>
+  </si>
+  <si>
+    <t>Por que senhas longas e difíceis são mais seguras do que senhas curtas e simples?</t>
+  </si>
+  <si>
+    <t>Porque são mais fáceis de lembrar</t>
+  </si>
+  <si>
+    <t>Porque programas usados por golpistas tentam adivinhar senhas automaticamente e senhas complexas levam muito mais tempo</t>
+  </si>
+  <si>
+    <t>Porque o celular exige senhas longas por padrão</t>
+  </si>
+  <si>
+    <t>Não faz diferença, qualquer senha é igualmente segura</t>
+  </si>
+  <si>
+    <t>Na verdade, senhas longas costumam ser mais difíceis de lembrar, mas são muito mais seguras.</t>
+  </si>
+  <si>
+    <t>Correto! Existem programas que tentam milhares de combinações de senha por segundo. Uma senha longa e complexa pode levar anos para ser descoberta.</t>
+  </si>
+  <si>
+    <t>O celular pode sugerir, mas a escolha é sempre sua. O motivo real é a segurança contra tentativas de invasão.</t>
+  </si>
+  <si>
+    <t>Faz muita diferença! Senhas como '123456' são descobertas em segundos. Uma senha longa e complexa é muito mais difícil de quebrar.</t>
+  </si>
+  <si>
+    <t>O que faz um aplicativo gerenciador de senhas?</t>
   </si>
 </sst>
 </file>
@@ -399,9 +653,11 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -735,8 +991,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{266F87BB-B8A9-4263-8D07-788549BAC926}">
-  <dimension ref="A1:K11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
@@ -752,389 +1008,739 @@
     <col min="11" max="11" width="112.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2">
         <v>3</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3">
         <v>2</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" t="s">
         <v>27</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
         <v>34</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4">
         <v>2</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" t="s">
         <v>36</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" t="s">
         <v>37</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" t="s">
         <v>38</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>41</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" t="s">
         <v>43</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5">
         <v>2</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" t="s">
         <v>45</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" t="s">
         <v>46</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" t="s">
         <v>47</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6">
         <v>3</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" t="s">
         <v>54</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" t="s">
         <v>55</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" t="s">
         <v>56</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="K6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>58</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s">
         <v>61</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" t="s">
         <v>62</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" t="s">
         <v>63</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7">
         <v>2</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" t="s">
         <v>64</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" t="s">
         <v>65</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" t="s">
         <v>66</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="K7" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>69</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" t="s">
         <v>70</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" t="s">
         <v>71</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" t="s">
         <v>72</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8">
         <v>3</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" t="s">
         <v>73</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" t="s">
         <v>74</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" t="s">
         <v>75</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="K8" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>78</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" t="s">
         <v>79</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" t="s">
         <v>80</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" t="s">
         <v>81</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9">
         <v>1</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" t="s">
         <v>82</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="I9" t="s">
         <v>83</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" t="s">
         <v>84</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="K9" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>87</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" t="s">
         <v>88</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" t="s">
         <v>89</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" t="s">
         <v>90</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10">
         <v>2</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H10" t="s">
         <v>91</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="I10" t="s">
         <v>92</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" t="s">
         <v>93</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="K10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>58</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>95</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>96</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" t="s">
         <v>97</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" t="s">
         <v>98</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" t="s">
         <v>99</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11">
         <v>2</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="H11" t="s">
         <v>100</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" t="s">
         <v>101</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" t="s">
         <v>102</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="K11" t="s">
         <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>104</v>
+      </c>
+      <c r="C12" t="s">
+        <v>105</v>
+      </c>
+      <c r="D12" t="s">
+        <v>106</v>
+      </c>
+      <c r="E12" t="s">
+        <v>107</v>
+      </c>
+      <c r="F12" t="s">
+        <v>108</v>
+      </c>
+      <c r="G12">
+        <v>2</v>
+      </c>
+      <c r="H12" t="s">
+        <v>109</v>
+      </c>
+      <c r="I12" t="s">
+        <v>110</v>
+      </c>
+      <c r="J12" t="s">
+        <v>111</v>
+      </c>
+      <c r="K12" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" t="s">
+        <v>115</v>
+      </c>
+      <c r="E13" t="s">
+        <v>116</v>
+      </c>
+      <c r="F13" t="s">
+        <v>117</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13" t="s">
+        <v>118</v>
+      </c>
+      <c r="I13" t="s">
+        <v>119</v>
+      </c>
+      <c r="J13" t="s">
+        <v>120</v>
+      </c>
+      <c r="K13" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C14" t="s">
+        <v>123</v>
+      </c>
+      <c r="D14" t="s">
+        <v>124</v>
+      </c>
+      <c r="E14" t="s">
+        <v>125</v>
+      </c>
+      <c r="F14" t="s">
+        <v>126</v>
+      </c>
+      <c r="G14">
+        <v>3</v>
+      </c>
+      <c r="H14" t="s">
+        <v>127</v>
+      </c>
+      <c r="I14" t="s">
+        <v>128</v>
+      </c>
+      <c r="J14" t="s">
+        <v>129</v>
+      </c>
+      <c r="K14" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C15" t="s">
+        <v>132</v>
+      </c>
+      <c r="D15" t="s">
+        <v>133</v>
+      </c>
+      <c r="E15" t="s">
+        <v>134</v>
+      </c>
+      <c r="F15" t="s">
+        <v>135</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15" t="s">
+        <v>136</v>
+      </c>
+      <c r="I15" t="s">
+        <v>137</v>
+      </c>
+      <c r="J15" t="s">
+        <v>138</v>
+      </c>
+      <c r="K15" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" t="s">
+        <v>140</v>
+      </c>
+      <c r="C16" t="s">
+        <v>141</v>
+      </c>
+      <c r="D16" t="s">
+        <v>142</v>
+      </c>
+      <c r="E16" t="s">
+        <v>143</v>
+      </c>
+      <c r="F16" t="s">
+        <v>144</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16" t="s">
+        <v>145</v>
+      </c>
+      <c r="I16" t="s">
+        <v>146</v>
+      </c>
+      <c r="J16" t="s">
+        <v>147</v>
+      </c>
+      <c r="K16" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" t="s">
+        <v>193</v>
+      </c>
+      <c r="C17" t="s">
+        <v>149</v>
+      </c>
+      <c r="D17" t="s">
+        <v>150</v>
+      </c>
+      <c r="E17" t="s">
+        <v>151</v>
+      </c>
+      <c r="F17" t="s">
+        <v>152</v>
+      </c>
+      <c r="G17">
+        <v>2</v>
+      </c>
+      <c r="H17" t="s">
+        <v>153</v>
+      </c>
+      <c r="I17" t="s">
+        <v>154</v>
+      </c>
+      <c r="J17" t="s">
+        <v>155</v>
+      </c>
+      <c r="K17" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" t="s">
+        <v>157</v>
+      </c>
+      <c r="C18" t="s">
+        <v>158</v>
+      </c>
+      <c r="D18" t="s">
+        <v>159</v>
+      </c>
+      <c r="E18" t="s">
+        <v>160</v>
+      </c>
+      <c r="F18" t="s">
+        <v>161</v>
+      </c>
+      <c r="G18">
+        <v>2</v>
+      </c>
+      <c r="H18" t="s">
+        <v>162</v>
+      </c>
+      <c r="I18" t="s">
+        <v>163</v>
+      </c>
+      <c r="J18" t="s">
+        <v>164</v>
+      </c>
+      <c r="K18" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" t="s">
+        <v>166</v>
+      </c>
+      <c r="C19" t="s">
+        <v>167</v>
+      </c>
+      <c r="D19" t="s">
+        <v>168</v>
+      </c>
+      <c r="E19" t="s">
+        <v>169</v>
+      </c>
+      <c r="F19" t="s">
+        <v>170</v>
+      </c>
+      <c r="G19">
+        <v>3</v>
+      </c>
+      <c r="H19" t="s">
+        <v>171</v>
+      </c>
+      <c r="I19" t="s">
+        <v>172</v>
+      </c>
+      <c r="J19" t="s">
+        <v>173</v>
+      </c>
+      <c r="K19" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" t="s">
+        <v>175</v>
+      </c>
+      <c r="C20" t="s">
+        <v>176</v>
+      </c>
+      <c r="D20" t="s">
+        <v>177</v>
+      </c>
+      <c r="E20" t="s">
+        <v>178</v>
+      </c>
+      <c r="F20" t="s">
+        <v>179</v>
+      </c>
+      <c r="G20">
+        <v>3</v>
+      </c>
+      <c r="H20" t="s">
+        <v>180</v>
+      </c>
+      <c r="I20" t="s">
+        <v>181</v>
+      </c>
+      <c r="J20" t="s">
+        <v>182</v>
+      </c>
+      <c r="K20" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" t="s">
+        <v>184</v>
+      </c>
+      <c r="C21" t="s">
+        <v>185</v>
+      </c>
+      <c r="D21" t="s">
+        <v>186</v>
+      </c>
+      <c r="E21" t="s">
+        <v>187</v>
+      </c>
+      <c r="F21" t="s">
+        <v>188</v>
+      </c>
+      <c r="G21">
+        <v>2</v>
+      </c>
+      <c r="H21" t="s">
+        <v>189</v>
+      </c>
+      <c r="I21" t="s">
+        <v>190</v>
+      </c>
+      <c r="J21" t="s">
+        <v>191</v>
+      </c>
+      <c r="K21" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>